<commit_message>
auto sync 2026-10-19 14:10:01
</commit_message>
<xml_diff>
--- a/Marathon_programme.xlsx
+++ b/Marathon_programme.xlsx
@@ -1882,9 +1882,11 @@
       <c r="G4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="6">
-        <f>"29' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n">
@@ -1922,9 +1924,12 @@
       <c r="G5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="6">
-        <f>"20' EF Z2 | 2x22' @ 91% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*91/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5' | 10' RC"&amp;CHAR(10)&amp;"FC bloc cible : ~165 bpm (85% FC max) | Cadence : 87-93 rpm"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"</f>
-        <v/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20' EF Z2 | 2x22' @ 91% FTP (180 W) — r=5' | 10' RC
+FC bloc cible : ~165 bpm (85% FC max) | Cadence : 87-93 rpm
+NUTRITION : 40g glucides/h si &gt;90'</t>
+        </is>
       </c>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n">
@@ -2045,9 +2050,11 @@
       <c r="G8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="6">
-        <f>"10' EF | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3' | 10' RC"&amp;CHAR(10)&amp;"FC : 131-155 bpm"</f>
-        <v/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10' EF | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3' | 10' RC
+FC : 131-155 bpm</t>
+        </is>
       </c>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n">
@@ -2335,9 +2342,11 @@
       <c r="G16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="6">
-        <f>"38' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n">
@@ -2375,9 +2384,14 @@
       <c r="G17" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H17" s="6">
-        <f>"20' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x10' @ 89% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*89/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~161 bpm (83% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20' EF Z2 (127-140 bpm / 120-140 W) | 2x10' @ 89% FTP (180 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~161 bpm (83% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n">
@@ -2457,9 +2471,13 @@
       <c r="G19" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="6">
-        <f>"10' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n">
@@ -2582,9 +2600,12 @@
       <c r="G22" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H22" s="6">
-        <f>"92' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 40g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n">
@@ -2785,9 +2806,11 @@
       <c r="G28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="6">
-        <f>"24' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n">
@@ -2825,9 +2848,14 @@
       <c r="G29" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H29" s="6">
-        <f>"20' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x9' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20' EF Z2 (127-140 bpm / 120-140 W) | 2x9' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n">
@@ -2950,9 +2978,13 @@
       <c r="G32" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H32" s="6">
-        <f>"10' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n">
@@ -3199,9 +3231,11 @@
       <c r="G39" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H39" s="6">
-        <f>"33' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n">
@@ -3239,9 +3273,14 @@
       <c r="G40" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="H40" s="6">
-        <f>"20' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x9' @ 92% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*92/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~167 bpm (86% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20' EF Z2 (127-140 bpm / 120-140 W) | 3x9' @ 92% FTP (185 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~167 bpm (86% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n">
@@ -3365,9 +3404,13 @@
       <c r="G43" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H43" s="6">
-        <f>"10' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n">
@@ -3490,9 +3533,12 @@
       <c r="G46" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H46" s="6">
-        <f>"94' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">94' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 40g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n">
@@ -3694,9 +3740,11 @@
       <c r="G52" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H52" s="6">
-        <f>"52' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n">
@@ -3734,9 +3782,14 @@
       <c r="G53" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H53" s="6">
-        <f>"89' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x7' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">89' EF Z2 (127-140 bpm / 120-140 W) | 2x7' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="n">
@@ -3861,9 +3914,13 @@
       <c r="G56" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H56" s="6">
-        <f>"39' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I56" s="3" t="n"/>
       <c r="J56" s="3" t="n">
@@ -4107,9 +4164,11 @@
       <c r="G63" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H63" s="6">
-        <f>"43' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I63" s="3" t="n"/>
       <c r="J63" s="3" t="n">
@@ -4147,9 +4206,14 @@
       <c r="G64" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H64" s="6">
-        <f>"45' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x12' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45' EF Z2 (127-140 bpm / 120-140 W) | 3x12' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I64" s="3" t="n"/>
       <c r="J64" s="3" t="n">
@@ -4278,9 +4342,13 @@
       <c r="G67" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H67" s="6">
-        <f>"50' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I67" s="3" t="n"/>
       <c r="J67" s="3" t="n">
@@ -4406,9 +4474,12 @@
       <c r="G70" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H70" s="6">
-        <f>"236' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">236' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 40g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I70" s="3" t="n"/>
       <c r="J70" s="3" t="n">
@@ -4610,9 +4681,11 @@
       <c r="G76" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H76" s="6">
-        <f>"43' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43' Z2 très facile (127-140 bpm / 100-120 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I76" s="3" t="n"/>
       <c r="J76" s="3" t="n">
@@ -4650,9 +4723,14 @@
       <c r="G77" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="H77" s="6">
-        <f>"51' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x12' over-unders : 3 x (3' @ 80% (155 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*93/500,0)*5,"0"),"?")&amp;" W"&amp;") + 1' @ 88% (171 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*107/500,0)*5,"0"),"?")&amp;" W"&amp;")) — r=5'"&amp;CHAR(10)&amp;"Objectif : tolérance au lactate et relances, alternance sous / au-dessus du seuil"&amp;CHAR(10)&amp;"FC : 155 bpm (80% FC max) sous le seuil | 171 bpm (88%) au-dessus (seuil lactique 163 bpm) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">51' EF Z2 (127-140 bpm / 120-140 W) | 3x12' over-unders : 3 x (3' @ 80% (155 bpm / 185 W) + 1' @ 88% (171 bpm / 215 W)) — r=5'
+Objectif : tolérance au lactate et relances, alternance sous / au-dessus du seuil
+FC : 155 bpm (80% FC max) sous le seuil | 171 bpm (88%) au-dessus (seuil lactique 163 bpm) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I77" s="3" t="n"/>
       <c r="J77" s="3" t="n">
@@ -4778,9 +4856,14 @@
       <c r="G80" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H80" s="6">
-        <f>"61' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I80" s="3" t="n"/>
       <c r="J80" s="3" t="n">
@@ -4906,9 +4989,12 @@
       <c r="G83" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H83" s="6">
-        <f>"246' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">246' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 40g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I83" s="3" t="n"/>
       <c r="J83" s="3" t="n">
@@ -5110,9 +5196,11 @@
       <c r="G89" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H89" s="6">
-        <f>"43' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I89" s="3" t="n"/>
       <c r="J89" s="3" t="n">
@@ -5150,9 +5238,14 @@
       <c r="G90" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="H90" s="6">
-        <f>"40' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3 ouvertures de 30'' à 90% FC max ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*120/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x3' @ 115% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*115/500,0)*5,"0"),"?")&amp;" W"&amp;" — 186 bpm en fin de répétition) — r=3' Z1 | 34' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Objectif : puissance aérobie maximale (VO2max), intervalles courts"&amp;CHAR(10)&amp;"FC fin de répétition : 184-194 bpm (95-100% FC max) | Cadence : 90-100 rpm | RPE 8-9/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40' EF Z2 (127-140 bpm / 120-140 W) dont 3 ouvertures de 30'' à 90% FC max (240 W) | 5x3' @ 115% FTP (230 W — 186 bpm en fin de répétition) — r=3' Z1 | 34' EF Z2 (127-140 bpm / 120-140 W)
+Objectif : puissance aérobie maximale (VO2max), intervalles courts
+FC fin de répétition : 184-194 bpm (95-100% FC max) | Cadence : 90-100 rpm | RPE 8-9/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I90" s="3" t="n"/>
       <c r="J90" s="3" t="n">
@@ -5278,9 +5371,14 @@
       <c r="G93" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H93" s="6">
-        <f>"72' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 40g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I93" s="3" t="n"/>
       <c r="J93" s="3" t="n">
@@ -5406,9 +5504,12 @@
       <c r="G96" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H96" s="6">
-        <f>"257' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 40g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">257' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 40g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I96" s="3" t="n"/>
       <c r="J96" s="3" t="n">
@@ -5610,9 +5711,11 @@
       <c r="G102" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H102" s="6">
-        <f>"32' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I102" s="3" t="n"/>
       <c r="J102" s="3" t="n">
@@ -5650,9 +5753,14 @@
       <c r="G103" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H103" s="6">
-        <f>"32' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x15' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32' EF Z2 (127-140 bpm / 120-140 W) | 2x15' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I103" s="3" t="n"/>
       <c r="J103" s="3" t="n">
@@ -5777,9 +5885,13 @@
       <c r="G106" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H106" s="6">
-        <f>"35' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I106" s="3" t="n"/>
       <c r="J106" s="3" t="n">
@@ -5905,9 +6017,13 @@
       <c r="G109" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H109" s="6">
-        <f>"167' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"Semaine deload — volume réduit"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">167' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+Semaine deload — volume réduit
+NUTRITION : 50g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I109" s="3" t="n"/>
       <c r="J109" s="3" t="n">
@@ -6071,9 +6187,11 @@
       <c r="G114" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H114" s="6">
-        <f>"43' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I114" s="3" t="n"/>
       <c r="J114" s="3" t="n">
@@ -6111,9 +6229,16 @@
       <c r="G115" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="H115" s="6">
-        <f>"25' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x1' rapide (110 rpm) | 5' très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") | 20' test — effort maximal régulier"&amp;CHAR(10)&amp;"Objectif : mesurer ta FTP (frais, après la semaine de décharge)"&amp;CHAR(10)&amp;"Départ : 5 premières minutes @ 100% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*100/500,0)*5,"0"),"?")&amp;" W"&amp;"), puis augmente de 5 W toutes les 5' si tu te sens bien — note la puissance moyenne des 20' et la FC moyenne des 10 dernières minutes | Cadence : 85-95 rpm | RPE 9/10"&amp;CHAR(10)&amp;"Calcul : FTP = 0,95 × puissance moyenne des 20' — à reporter dans la case FTP de l'onglet Repères vélo"&amp;CHAR(10)&amp;"56' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H115" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25' EF Z2 (127-140 bpm / 120-140 W) dont 3x1' rapide (110 rpm) | 5' très facile (127-140 bpm / 100-120 W) | 20' test — effort maximal régulier
+Objectif : mesurer ta FTP (frais, après la semaine de décharge)
+Départ : 5 premières minutes @ 100% FTP (200 W), puis augmente de 5 W toutes les 5' si tu te sens bien — note la puissance moyenne des 20' et la FC moyenne des 10 dernières minutes | Cadence : 85-95 rpm | RPE 9/10
+Calcul : FTP = 0,95 × puissance moyenne des 20' — à reporter dans la case FTP de l'onglet Repères vélo
+56' EF Z2 (127-140 bpm / 120-140 W)
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I115" s="3" t="n"/>
       <c r="J115" s="3" t="n">
@@ -6240,9 +6365,14 @@
       <c r="G118" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H118" s="6">
-        <f>"70' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H118" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I118" s="3" t="n"/>
       <c r="J118" s="3" t="n">
@@ -6368,9 +6498,12 @@
       <c r="G121" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H121" s="6">
-        <f>"261' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H121" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">261' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 50g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I121" s="3" t="n"/>
       <c r="J121" s="3" t="n">
@@ -6579,9 +6712,11 @@
       <c r="G127" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H127" s="6">
-        <f>"43' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H127" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I127" s="3" t="n"/>
       <c r="J127" s="3" t="n">
@@ -6619,9 +6754,14 @@
       <c r="G128" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="H128" s="6">
-        <f>"64' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x9' @ 102% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*102/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=4'"&amp;CHAR(10)&amp;"Objectif : élever le seuil (blocs courts à intensité haute)"&amp;CHAR(10)&amp;"FC bloc cible : ~169 bpm (87% FC max, 6 bpm au-dessus de ton seuil lactique de 163) | Cadence : 88-95 rpm | RPE 8/10"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">64' EF Z2 (127-140 bpm / 120-140 W) | 4x9' @ 102% FTP (205 W) — r=4'
+Objectif : élever le seuil (blocs courts à intensité haute)
+FC bloc cible : ~169 bpm (87% FC max, 6 bpm au-dessus de ton seuil lactique de 163) | Cadence : 88-95 rpm | RPE 8/10
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I128" s="3" t="n"/>
       <c r="J128" s="3" t="n">
@@ -6747,9 +6887,14 @@
       <c r="G131" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H131" s="6">
-        <f>"72' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H131" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I131" s="3" t="n"/>
       <c r="J131" s="3" t="n">
@@ -6875,9 +7020,12 @@
       <c r="G134" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H134" s="6">
-        <f>"268' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">268' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 50g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I134" s="3" t="n"/>
       <c r="J134" s="3" t="n">
@@ -7081,9 +7229,11 @@
       <c r="G140" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H140" s="6">
-        <f>"47' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I140" s="3" t="n"/>
       <c r="J140" s="3" t="n">
@@ -7121,9 +7271,14 @@
       <c r="G141" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="H141" s="6">
-        <f>"71' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x20' over-unders : 5 x (3' @ 93% FTP (~155 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*93/500,0)*5,"0"),"?")&amp;" W"&amp;") + 1' @ 107% FTP (~171 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*107/500,0)*5,"0"),"?")&amp;" W"&amp;")) — r=5'"&amp;CHAR(10)&amp;"Objectif : tolérance au lactate et relances, alternance sous / au-dessus du seuil"&amp;CHAR(10)&amp;"FC : 155 bpm (80% FC max) sous le seuil | 171 bpm (88%) au-dessus (seuil lactique 163 bpm) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H141" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71' EF Z2 (127-140 bpm / 120-140 W) | 2x20' over-unders : 5 x (3' @ 93% FTP (~155 bpm / 185 W) + 1' @ 107% FTP (~171 bpm / 215 W)) — r=5'
+Objectif : tolérance au lactate et relances, alternance sous / au-dessus du seuil
+FC : 155 bpm (80% FC max) sous le seuil | 171 bpm (88%) au-dessus (seuil lactique 163 bpm) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I141" s="3" t="n"/>
       <c r="J141" s="3" t="n">
@@ -7249,9 +7404,14 @@
       <c r="G144" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H144" s="6">
-        <f>"74' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H144" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 50g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I144" s="3" t="n"/>
       <c r="J144" s="3" t="n">
@@ -7378,9 +7538,12 @@
       <c r="G147" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H147" s="6">
-        <f>"274' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 50g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H147" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">274' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 50g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I147" s="3" t="n"/>
       <c r="J147" s="3" t="n">
@@ -7584,9 +7747,11 @@
       <c r="G153" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H153" s="6">
-        <f>"32' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H153" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I153" s="3" t="n"/>
       <c r="J153" s="3" t="n">
@@ -7624,9 +7789,14 @@
       <c r="G154" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H154" s="6">
-        <f>"30' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x18' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H154" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30' EF Z2 (127-140 bpm / 120-140 W) | 2x18' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I154" s="3" t="n"/>
       <c r="J154" s="3" t="n">
@@ -7752,9 +7922,13 @@
       <c r="G157" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H157" s="6">
-        <f>"42' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H157" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">42' EF (127-140 bpm / 120-140 W) | 4x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I157" s="3" t="n"/>
       <c r="J157" s="3" t="n">
@@ -7879,9 +8053,13 @@
       <c r="G160" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H160" s="6">
-        <f>"182' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"Semaine deload — volume réduit"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H160" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">182' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+Semaine deload — volume réduit
+NUTRITION : 60g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I160" s="3" t="n"/>
       <c r="J160" s="3" t="n">
@@ -8040,9 +8218,11 @@
       <c r="G165" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H165" s="6">
-        <f>"47' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H165" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I165" s="3" t="n"/>
       <c r="J165" s="3" t="n">
@@ -8080,9 +8260,14 @@
       <c r="G166" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H166" s="6">
-        <f>"61' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x25' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H166" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61' EF Z2 (127-140 bpm / 120-140 W) | 2x25' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I166" s="3" t="n"/>
       <c r="J166" s="3" t="n">
@@ -8251,9 +8436,14 @@
       <c r="G170" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H170" s="6">
-        <f>"74' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H170" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I170" s="3" t="n"/>
       <c r="J170" s="3" t="n">
@@ -8380,9 +8570,12 @@
       <c r="G173" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H173" s="6">
-        <f>"279' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">279' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 60g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I173" s="3" t="n"/>
       <c r="J173" s="3" t="n">
@@ -8591,9 +8784,11 @@
       <c r="G179" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H179" s="6">
-        <f>"47' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H179" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I179" s="3" t="n"/>
       <c r="J179" s="3" t="n">
@@ -8631,9 +8826,14 @@
       <c r="G180" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="H180" s="6">
-        <f>"40' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3 ouvertures de 30'' à 90% FC max ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*120/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' @ 112% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*112/500,0)*5,"0"),"?")&amp;" W"&amp;" — 186 bpm en fin de répétition) — r=4' Z1 | 51' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Objectif : puissance aérobie maximale (VO2max), intervalles courts"&amp;CHAR(10)&amp;"FC fin de répétition : 184-194 bpm (95-100% FC max) | Cadence : 90-100 rpm | RPE 8-9/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H180" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40' EF Z2 (127-140 bpm / 120-140 W) dont 3 ouvertures de 30'' à 90% FC max (240 W) | 5x4' @ 112% FTP (225 W — 186 bpm en fin de répétition) — r=4' Z1 | 51' EF Z2 (127-140 bpm / 120-140 W)
+Objectif : puissance aérobie maximale (VO2max), intervalles courts
+FC fin de répétition : 184-194 bpm (95-100% FC max) | Cadence : 90-100 rpm | RPE 8-9/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I180" s="3" t="n"/>
       <c r="J180" s="3" t="n">
@@ -8801,9 +9001,14 @@
       <c r="G184" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H184" s="6">
-        <f>"79' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H184" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I184" s="3" t="n"/>
       <c r="J184" s="3" t="n">
@@ -8930,9 +9135,12 @@
       <c r="G187" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H187" s="6">
-        <f>"285' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H187" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">285' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 60g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I187" s="3" t="n"/>
       <c r="J187" s="3" t="n">
@@ -9137,9 +9345,11 @@
       <c r="G193" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H193" s="6">
-        <f>"51' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H193" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">51' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I193" s="3" t="n"/>
       <c r="J193" s="3" t="n">
@@ -9177,9 +9387,14 @@
       <c r="G194" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H194" s="6">
-        <f>"66' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x20' à 147-159 bpm (76-82% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*82/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*87/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : endurance de tempo, pont vers l'allure IM"&amp;CHAR(10)&amp;"FC bloc cible : 147-159 bpm (76-82% FC max) | Cadence : 85-92 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H194" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">66' EF Z2 (127-140 bpm / 120-140 W) | 3x20' à 147-159 bpm (76-82% FC max / 165-175 W) — r=5'
+Objectif : endurance de tempo, pont vers l'allure IM
+FC bloc cible : 147-159 bpm (76-82% FC max) | Cadence : 85-92 rpm | RPE 6-7/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I194" s="3" t="n"/>
       <c r="J194" s="3" t="n">
@@ -9347,9 +9562,14 @@
       <c r="G198" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H198" s="6">
-        <f>"83' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H198" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">83' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I198" s="3" t="n"/>
       <c r="J198" s="3" t="n">
@@ -9476,9 +9696,12 @@
       <c r="G201" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H201" s="6">
-        <f>"289' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H201" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">289' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 60g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I201" s="3" t="n"/>
       <c r="J201" s="3" t="n">
@@ -9635,9 +9858,14 @@
       <c r="G206" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H206" s="6">
-        <f>"70' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x12' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H206" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70' EF Z2 (127-140 bpm / 120-140 W) | 2x12' @ 90% FTP (180 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~163 bpm (84% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 60g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I206" s="3" t="n"/>
       <c r="J206" s="3" t="n">
@@ -9721,9 +9949,12 @@
       <c r="G208" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H208" s="6">
-        <f>"100' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") — parcours Paris, terrain plat"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;90'"</f>
-        <v/>
+      <c r="H208" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100' Z2 (127-140 bpm / 120-140 W) — parcours Paris, terrain plat
+Cadence souple 85-90 rpm
+NUTRITION : 60g glucides/h si &gt;90'</t>
+        </is>
       </c>
       <c r="I208" s="3" t="n"/>
       <c r="J208" s="3" t="n">
@@ -10361,9 +10592,11 @@
       <c r="G224" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H224" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H224" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I224" s="3" t="n"/>
       <c r="J224" s="3" t="n">
@@ -10401,9 +10634,12 @@
       <c r="G225" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H225" s="6">
-        <f>"193' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 60g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H225" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">193' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 60g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I225" s="3" t="n"/>
       <c r="J225" s="3" t="n">
@@ -10647,9 +10883,11 @@
       <c r="G232" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H232" s="6">
-        <f>"51' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H232" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">51' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I232" s="3" t="n"/>
       <c r="J232" s="3" t="n">
@@ -10687,9 +10925,14 @@
       <c r="G233" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H233" s="6">
-        <f>"53' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x28' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H233" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">53' EF Z2 (127-140 bpm / 120-140 W) | 2x28' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I233" s="3" t="n"/>
       <c r="J233" s="3" t="n">
@@ -10859,9 +11102,14 @@
       <c r="G237" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H237" s="6">
-        <f>"61' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H237" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I237" s="3" t="n"/>
       <c r="J237" s="3" t="n">
@@ -10988,9 +11236,12 @@
       <c r="G240" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H240" s="6">
-        <f>"257' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H240" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">257' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 70g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I240" s="3" t="n"/>
       <c r="J240" s="3" t="n">
@@ -11237,9 +11488,11 @@
       <c r="G247" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H247" s="6">
-        <f>"51' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H247" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">51' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I247" s="3" t="n"/>
       <c r="J247" s="3" t="n">
@@ -11277,9 +11530,14 @@
       <c r="G248" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H248" s="6">
-        <f>"56' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x30' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H248" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56' EF Z2 (127-140 bpm / 120-140 W) | 2x30' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I248" s="3" t="n"/>
       <c r="J248" s="3" t="n">
@@ -11446,9 +11704,14 @@
       <c r="G252" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H252" s="6">
-        <f>"65' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H252" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">65' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I252" s="3" t="n"/>
       <c r="J252" s="3" t="n">
@@ -11575,9 +11838,12 @@
       <c r="G255" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H255" s="6">
-        <f>"279' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H255" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">279' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 70g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I255" s="3" t="n"/>
       <c r="J255" s="3" t="n">
@@ -11824,9 +12090,11 @@
       <c r="G262" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H262" s="6">
-        <f>"54' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H262" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I262" s="3" t="n"/>
       <c r="J262" s="3" t="n">
@@ -11864,9 +12132,14 @@
       <c r="G263" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H263" s="6">
-        <f>"62' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x30' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H263" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62' EF Z2 (127-140 bpm / 120-140 W) | 2x30' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I263" s="3" t="n"/>
       <c r="J263" s="3" t="n">
@@ -12034,9 +12307,14 @@
       <c r="G267" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H267" s="6">
-        <f>"72' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H267" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I267" s="3" t="n"/>
       <c r="J267" s="3" t="n">
@@ -12163,9 +12441,12 @@
       <c r="G270" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H270" s="6">
-        <f>"296' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H270" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">296' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 70g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I270" s="3" t="n"/>
       <c r="J270" s="3" t="n">
@@ -12413,9 +12694,11 @@
       <c r="G277" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H277" s="6">
-        <f>"39' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H277" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I277" s="3" t="n"/>
       <c r="J277" s="3" t="n">
@@ -12453,9 +12736,14 @@
       <c r="G278" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H278" s="6">
-        <f>"35' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x20' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H278" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35' EF Z2 (127-140 bpm / 120-140 W) | 2x20' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I278" s="3" t="n"/>
       <c r="J278" s="3" t="n">
@@ -12622,9 +12910,13 @@
       <c r="G282" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H282" s="6">
-        <f>"40' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H282" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I282" s="3" t="n"/>
       <c r="J282" s="3" t="n">
@@ -12750,9 +13042,13 @@
       <c r="G285" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H285" s="6">
-        <f>"193' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"Semaine deload — volume réduit"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H285" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">193' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+Semaine deload — volume réduit
+NUTRITION : 70g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I285" s="3" t="n"/>
       <c r="J285" s="3" t="n">
@@ -12951,9 +13247,11 @@
       <c r="G291" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H291" s="6">
-        <f>"54' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H291" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I291" s="3" t="n"/>
       <c r="J291" s="3" t="n">
@@ -12991,9 +13289,16 @@
       <c r="G292" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="H292" s="6">
-        <f>"25' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x1' rapide (110 rpm) | 5' très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") | 20' test — effort maximal régulier"&amp;CHAR(10)&amp;"Objectif : mesurer ta FTP (frais, après la semaine de décharge)"&amp;CHAR(10)&amp;"Départ : 5 premières minutes @ 100% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*100/500,0)*5,"0"),"?")&amp;" W"&amp;"), puis augmente de 5 W toutes les 5' si tu te sens bien — note la puissance moyenne des 20' et la FC moyenne des 10 dernières minutes | Cadence : 85-95 rpm | RPE 9/10"&amp;CHAR(10)&amp;"Calcul : FTP = 0,95 × puissance moyenne des 20' — à reporter dans la case FTP de l'onglet Repères vélo"&amp;CHAR(10)&amp;"81' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H292" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25' EF Z2 (127-140 bpm / 120-140 W) dont 3x1' rapide (110 rpm) | 5' très facile (127-140 bpm / 100-120 W) | 20' test — effort maximal régulier
+Objectif : mesurer ta FTP (frais, après la semaine de décharge)
+Départ : 5 premières minutes @ 100% FTP (200 W), puis augmente de 5 W toutes les 5' si tu te sens bien — note la puissance moyenne des 20' et la FC moyenne des 10 dernières minutes | Cadence : 85-95 rpm | RPE 9/10
+Calcul : FTP = 0,95 × puissance moyenne des 20' — à reporter dans la case FTP de l'onglet Repères vélo
+81' EF Z2 (127-140 bpm / 120-140 W)
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I292" s="3" t="n"/>
       <c r="J292" s="3" t="n">
@@ -13160,9 +13465,14 @@
       <c r="G296" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H296" s="6">
-        <f>"74' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H296" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I296" s="3" t="n"/>
       <c r="J296" s="3" t="n">
@@ -13289,9 +13599,12 @@
       <c r="G299" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H299" s="6">
-        <f>"300' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H299" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">300' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 70g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I299" s="3" t="n"/>
       <c r="J299" s="3" t="n">
@@ -13535,9 +13848,11 @@
       <c r="G306" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H306" s="6">
-        <f>"56' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H306" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I306" s="3" t="n"/>
       <c r="J306" s="3" t="n">
@@ -13620,9 +13935,14 @@
       <c r="G308" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="H308" s="6">
-        <f>"40' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3 ouvertures de 30'' à 90% FC max ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*120/500,0)*5,"0"),"?")&amp;" W"&amp;") | 6x4' @ 112% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*112/500,0)*5,"0"),"?")&amp;" W"&amp;" — 186 bpm en fin de répétition) — r=4' Z1 | 56' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Objectif : puissance aérobie maximale (VO2max), intervalles courts"&amp;CHAR(10)&amp;"FC fin de répétition : 184-194 bpm (95-100% FC max) | Cadence : 90-100 rpm | RPE 8-9/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H308" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40' EF Z2 (127-140 bpm / 120-140 W) dont 3 ouvertures de 30'' à 90% FC max (240 W) | 6x4' @ 112% FTP (225 W — 186 bpm en fin de répétition) — r=4' Z1 | 56' EF Z2 (127-140 bpm / 120-140 W)
+Objectif : puissance aérobie maximale (VO2max), intervalles courts
+FC fin de répétition : 184-194 bpm (95-100% FC max) | Cadence : 90-100 rpm | RPE 8-9/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I308" s="3" t="n"/>
       <c r="J308" s="3" t="n">
@@ -13789,9 +14109,14 @@
       <c r="G312" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H312" s="6">
-        <f>"80' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H312" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 70g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I312" s="3" t="n"/>
       <c r="J312" s="3" t="n">
@@ -13872,9 +14197,12 @@
       <c r="G314" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H314" s="6">
-        <f>"311' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 70g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H314" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">311' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 70g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I314" s="3" t="n"/>
       <c r="J314" s="3" t="n">
@@ -14034,9 +14362,11 @@
       <c r="G319" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H319" s="6">
-        <f>"58' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H319" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">58' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I319" s="3" t="n"/>
       <c r="J319" s="3" t="n">
@@ -14074,9 +14404,14 @@
       <c r="G320" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H320" s="6">
-        <f>"78' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x33' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H320" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78' EF Z2 (127-140 bpm / 120-140 W) | 2x33' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I320" s="3" t="n"/>
       <c r="J320" s="3" t="n">
@@ -14244,9 +14579,14 @@
       <c r="G324" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H324" s="6">
-        <f>"89' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H324" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">89' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I324" s="3" t="n"/>
       <c r="J324" s="3" t="n">
@@ -14373,9 +14713,12 @@
       <c r="G327" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H327" s="6">
-        <f>"321' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H327" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">321' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 80g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I327" s="3" t="n"/>
       <c r="J327" s="3" t="n">
@@ -14623,9 +14966,11 @@
       <c r="G334" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H334" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H334" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I334" s="3" t="n"/>
       <c r="J334" s="3" t="n">
@@ -14663,9 +15008,14 @@
       <c r="G335" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H335" s="6">
-        <f>"72' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x40' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H335" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72' EF Z2 (127-140 bpm / 120-140 W) | 2x40' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I335" s="3" t="n"/>
       <c r="J335" s="3" t="n">
@@ -14833,9 +15183,14 @@
       <c r="G339" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H339" s="6">
-        <f>"95' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H339" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">95' EF (127-140 bpm / 120-140 W) | 5x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I339" s="3" t="n"/>
       <c r="J339" s="3" t="n">
@@ -14962,9 +15317,12 @@
       <c r="G342" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H342" s="6">
-        <f>"332' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H342" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">332' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 80g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I342" s="3" t="n"/>
       <c r="J342" s="3" t="n">
@@ -15529,9 +15887,11 @@
       <c r="G358" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H358" s="6">
-        <f>"51' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H358" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">51' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I358" s="3" t="n"/>
       <c r="J358" s="3" t="n">
@@ -15569,9 +15929,12 @@
       <c r="G359" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H359" s="6">
-        <f>"120' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") — pas de bloc FTP cette semaine (reprise post-ski)"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"</f>
-        <v/>
+      <c r="H359" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120' Z2 (127-140 bpm / 120-140 W) — pas de bloc FTP cette semaine (reprise post-ski)
+Cadence souple 85-90 rpm
+NUTRITION : 80g glucides/h si &gt;90'</t>
+        </is>
       </c>
       <c r="I359" s="3" t="n"/>
       <c r="J359" s="3" t="n">
@@ -15738,9 +16101,12 @@
       <c r="G363" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H363" s="6">
-        <f>"96' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — pas de travail de force cette semaine"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"</f>
-        <v/>
+      <c r="H363" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96' Z2 très facile (127-140 bpm / 100-120 W) — pas de travail de force cette semaine
+Cadence souple 85-90 rpm
+NUTRITION : 80g glucides/h si &gt;90'</t>
+        </is>
       </c>
       <c r="I363" s="3" t="n"/>
       <c r="J363" s="3" t="n">
@@ -15867,9 +16233,12 @@
       <c r="G366" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H366" s="6">
-        <f>"246' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H366" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">246' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 80g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I366" s="3" t="n"/>
       <c r="J366" s="3" t="n">
@@ -16116,9 +16485,11 @@
       <c r="G373" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H373" s="6">
-        <f>"56' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H373" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I373" s="3" t="n"/>
       <c r="J373" s="3" t="n">
@@ -16156,9 +16527,14 @@
       <c r="G374" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H374" s="6">
-        <f>"66' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x30' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H374" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">66' EF Z2 (127-140 bpm / 120-140 W) | 2x30' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I374" s="3" t="n"/>
       <c r="J374" s="3" t="n">
@@ -16328,9 +16704,14 @@
       <c r="G378" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H378" s="6">
-        <f>"77' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H378" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77' EF (127-140 bpm / 120-140 W) | 5x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I378" s="3" t="n"/>
       <c r="J378" s="3" t="n">
@@ -16457,9 +16838,12 @@
       <c r="G381" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H381" s="6">
-        <f>"300' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H381" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">300' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 80g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I381" s="3" t="n"/>
       <c r="J381" s="3" t="n">
@@ -16707,9 +17091,11 @@
       <c r="G388" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H388" s="6">
-        <f>"47' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H388" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I388" s="3" t="n"/>
       <c r="J388" s="3" t="n">
@@ -16747,9 +17133,14 @@
       <c r="G389" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H389" s="6">
-        <f>"52' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x20' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H389" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52' EF Z2 (127-140 bpm / 120-140 W) | 2x20' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I389" s="3" t="n"/>
       <c r="J389" s="3" t="n">
@@ -16916,9 +17307,13 @@
       <c r="G393" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H393" s="6">
-        <f>"46' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H393" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">46' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I393" s="3" t="n"/>
       <c r="J393" s="3" t="n">
@@ -17045,9 +17440,13 @@
       <c r="G396" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H396" s="6">
-        <f>"236' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"Semaine deload — volume réduit"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H396" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">236' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+Semaine deload — volume réduit
+NUTRITION : 80g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I396" s="3" t="n"/>
       <c r="J396" s="3" t="n">
@@ -17249,9 +17648,11 @@
       <c r="G402" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H402" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H402" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I402" s="3" t="n"/>
       <c r="J402" s="3" t="n">
@@ -17289,9 +17690,14 @@
       <c r="G403" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H403" s="6">
-        <f>"61' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x25' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H403" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61' EF Z2 (127-140 bpm / 120-140 W) | 3x25' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I403" s="3" t="n"/>
       <c r="J403" s="3" t="n">
@@ -17459,9 +17865,14 @@
       <c r="G407" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H407" s="6">
-        <f>"79' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H407" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79' EF (127-140 bpm / 120-140 W) | 5x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 80g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I407" s="3" t="n"/>
       <c r="J407" s="3" t="n">
@@ -17588,9 +17999,12 @@
       <c r="G410" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H410" s="6">
-        <f>"321' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 80g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H410" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">321' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 80g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I410" s="3" t="n"/>
       <c r="J410" s="3" t="n">
@@ -17837,9 +18251,11 @@
       <c r="G417" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H417" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H417" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I417" s="3" t="n"/>
       <c r="J417" s="3" t="n">
@@ -17877,9 +18293,14 @@
       <c r="G418" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H418" s="6">
-        <f>"106' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x25' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : travailler juste sous le seuil lactique (sweet spot)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H418" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">106' EF Z2 (127-140 bpm / 120-140 W) | 2x25' @ 90% FTP (180 W) — r=5'
+Objectif : travailler juste sous le seuil lactique (sweet spot)
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I418" s="3" t="n"/>
       <c r="J418" s="3" t="n">
@@ -18047,9 +18468,14 @@
       <c r="G422" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H422" s="6">
-        <f>"86' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H422" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">86' EF (127-140 bpm / 120-140 W) | 5x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I422" s="3" t="n"/>
       <c r="J422" s="3" t="n">
@@ -18176,9 +18602,12 @@
       <c r="G425" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H425" s="6">
-        <f>"343' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H425" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">343' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I425" s="3" t="n"/>
       <c r="J425" s="3" t="n">
@@ -18425,9 +18854,11 @@
       <c r="G432" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H432" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H432" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I432" s="3" t="n"/>
       <c r="J432" s="3" t="n">
@@ -18465,9 +18896,14 @@
       <c r="G433" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H433" s="6">
-        <f>"100' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x20' à 147-159 bpm (76-82% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*82/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*87/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : endurance de tempo, pont vers l'allure IM"&amp;CHAR(10)&amp;"FC bloc cible : 147-159 bpm (76-82% FC max) | Cadence : 85-92 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H433" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100' EF Z2 (127-140 bpm / 120-140 W) | 3x20' à 147-159 bpm (76-82% FC max / 165-175 W) — r=5'
+Objectif : endurance de tempo, pont vers l'allure IM
+FC bloc cible : 147-159 bpm (76-82% FC max) | Cadence : 85-92 rpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I433" s="3" t="n"/>
       <c r="J433" s="3" t="n">
@@ -18635,9 +19071,14 @@
       <c r="G437" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H437" s="6">
-        <f>"99' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 5x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H437" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">99' EF (127-140 bpm / 120-140 W) | 5x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I437" s="3" t="n"/>
       <c r="J437" s="3" t="n">
@@ -18764,9 +19205,12 @@
       <c r="G440" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H440" s="6">
-        <f>"364' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H440" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">364' Z2 (127-140 bpm / 120-140 W)
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I440" s="3" t="n"/>
       <c r="J440" s="3" t="n">
@@ -19010,9 +19454,11 @@
       <c r="G447" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H447" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H447" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I447" s="3" t="n"/>
       <c r="J447" s="3" t="n">
@@ -19050,9 +19496,14 @@
       <c r="G448" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H448" s="6">
-        <f>"67' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x25' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : rester juste sous le seuil lactique, séance complète — Lacanau est une course en Z3, pas d'affûtage"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H448" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">67' EF Z2 (127-140 bpm / 120-140 W) | 2x25' @ 90% FTP (180 W) — r=5'
+Objectif : rester juste sous le seuil lactique, séance complète — Lacanau est une course en Z3, pas d'affûtage
+FC bloc cible : ~163 bpm (84% FC max = ton seuil lactique) | Cadence : 87-93 rpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I448" s="3" t="n"/>
       <c r="J448" s="3" t="n">
@@ -19219,9 +19670,13 @@
       <c r="G452" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H452" s="6">
-        <f>"26' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H452" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26' EF (127-140 bpm / 120-140 W) | 3x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I452" s="3" t="n"/>
       <c r="J452" s="3" t="n">
@@ -19345,9 +19800,10 @@
       <c r="G455" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H455" s="6">
-        <f>"15' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — vérification matériel / dépôt sac T1-T2"</f>
-        <v/>
+      <c r="H455" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15' Z2 très facile (127-140 bpm / 100-120 W) — vérification matériel / dépôt sac T1-T2</t>
+        </is>
       </c>
       <c r="I455" s="3" t="n"/>
       <c r="J455" s="3" t="n">
@@ -19560,9 +20016,11 @@
       <c r="G461" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H461" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H461" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I461" s="3" t="n"/>
       <c r="J461" s="3" t="n">
@@ -19600,9 +20058,12 @@
       <c r="G462" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H462" s="6">
-        <f>"118' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") — Z2 facile, pas de bloc FTP (reprise post-Lacanau)"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"</f>
-        <v/>
+      <c r="H462" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">118' Z2 (127-140 bpm / 120-140 W) — Z2 facile, pas de bloc FTP (reprise post-Lacanau)
+Cadence souple 85-90 rpm
+NUTRITION : 90g glucides/h si &gt;90'</t>
+        </is>
       </c>
       <c r="I462" s="3" t="n"/>
       <c r="J462" s="3" t="n">
@@ -19769,9 +20230,11 @@
       <c r="G466" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H466" s="6">
-        <f>"75' Z2 facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H466" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75' Z2 facile (127-140 bpm / 120-140 W)
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I466" s="3" t="n"/>
       <c r="J466" s="3" t="n">
@@ -19855,9 +20318,11 @@
       <c r="G468" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H468" s="6">
-        <f>"214' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — Z2 léger, reprise du volume"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"</f>
-        <v/>
+      <c r="H468" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">214' Z2 (127-140 bpm / 100-120 W) — Z2 léger, reprise du volume
+NUTRITION : 90g glucides/h si &gt;90'</t>
+        </is>
       </c>
       <c r="I468" s="3" t="n"/>
       <c r="J468" s="3" t="n">
@@ -20112,9 +20577,11 @@
       <c r="G475" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H475" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H475" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I475" s="3" t="n"/>
       <c r="J475" s="3" t="n">
@@ -20152,9 +20619,14 @@
       <c r="G476" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H476" s="6">
-        <f>"85' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x25' @ 90% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*90/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : reprendre le développement du seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~163 bpm (84% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H476" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">85' EF Z2 (127-140 bpm / 120-140 W) | 2x25' @ 90% FTP (180 W) — r=5'
+Objectif : reprendre le développement du seuil (FTP)
+FC bloc cible : ~163 bpm (84% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I476" s="3" t="n"/>
       <c r="J476" s="3" t="n">
@@ -20322,9 +20794,14 @@
       <c r="G480" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H480" s="6">
-        <f>"87' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H480" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I480" s="3" t="n"/>
       <c r="J480" s="3" t="n">
@@ -20451,9 +20928,12 @@
       <c r="G483" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H483" s="6">
-        <f>"321' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 2x30' allure IM (136-146 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") dans la seconde moitié — r=10' Z2"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H483" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">321' Z2 (127-140 bpm / 120-140 W) dont 2x30' allure IM (136-146 bpm / 140-150 W) dans la seconde moitié — r=10' Z2
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I483" s="3" t="n"/>
       <c r="J483" s="3" t="n">
@@ -20707,9 +21187,11 @@
       <c r="G490" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H490" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H490" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I490" s="3" t="n"/>
       <c r="J490" s="3" t="n">
@@ -20747,9 +21229,14 @@
       <c r="G491" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H491" s="6">
-        <f>"69' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x35' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H491" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">69' EF Z2 (127-140 bpm / 120-140 W) | 2x35' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I491" s="3" t="n"/>
       <c r="J491" s="3" t="n">
@@ -20916,9 +21403,14 @@
       <c r="G495" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H495" s="6">
-        <f>"74' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 6x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H495" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74' EF (127-140 bpm / 120-140 W) | 6x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I495" s="3" t="n"/>
       <c r="J495" s="3" t="n">
@@ -21045,9 +21537,12 @@
       <c r="G498" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H498" s="6">
-        <f>"343' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x30' allure IM (136-146 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") dans la seconde moitié — r=10' Z2"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H498" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">343' Z2 (127-140 bpm / 120-140 W) dont 3x30' allure IM (136-146 bpm / 140-150 W) dans la seconde moitié — r=10' Z2
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I498" s="3" t="n"/>
       <c r="J498" s="3" t="n">
@@ -21302,9 +21797,11 @@
       <c r="G505" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H505" s="6">
-        <f>"43' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H505" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I505" s="3" t="n"/>
       <c r="J505" s="3" t="n">
@@ -21342,9 +21839,14 @@
       <c r="G506" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H506" s="6">
-        <f>"33' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x22' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : développer la puissance au seuil (FTP)"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H506" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33' EF Z2 (127-140 bpm / 120-140 W) | 2x22' @ 88% FTP (175 W) — r=5'
+Objectif : développer la puissance au seuil (FTP)
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I506" s="3" t="n"/>
       <c r="J506" s="3" t="n">
@@ -21511,9 +22013,13 @@
       <c r="G510" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H510" s="6">
-        <f>"42' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 4x4' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H510" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">42' EF (127-140 bpm / 120-140 W) | 4x4' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I510" s="3" t="n"/>
       <c r="J510" s="3" t="n">
@@ -21595,9 +22101,12 @@
       <c r="G512" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="H512" s="6">
-        <f>"300' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x40' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;")"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h — stratégie course complète"</f>
-        <v/>
+      <c r="H512" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">300' Z2 (127-140 bpm / 120-140 W) dont 3x40' allure IM (136-146 bpm, 70-75% FC max / 140-150 W)
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h — stratégie course complète</t>
+        </is>
       </c>
       <c r="I512" s="3" t="n"/>
       <c r="J512" s="3" t="n">
@@ -21844,9 +22353,11 @@
       <c r="G519" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H519" s="6">
-        <f>"64' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H519" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">64' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I519" s="3" t="n"/>
       <c r="J519" s="3" t="n">
@@ -21929,9 +22440,14 @@
       <c r="G521" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H521" s="6">
-        <f>"53' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x30' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H521" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">53' EF Z2 (127-140 bpm / 120-140 W) | 3x30' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I521" s="3" t="n"/>
       <c r="J521" s="3" t="n">
@@ -22098,9 +22614,14 @@
       <c r="G525" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H525" s="6">
-        <f>"78' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 6x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H525" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78' EF (127-140 bpm / 120-140 W) | 6x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I525" s="3" t="n"/>
       <c r="J525" s="3" t="n">
@@ -22226,9 +22747,12 @@
       <c r="G528" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H528" s="6">
-        <f>"354' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x40' allure IM (136-146 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") dans la seconde moitié — r=10' Z2"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H528" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">354' Z2 (127-140 bpm / 120-140 W) dont 3x40' allure IM (136-146 bpm / 140-150 W) dans la seconde moitié — r=10' Z2
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I528" s="3" t="n"/>
       <c r="J528" s="3" t="n">
@@ -22431,9 +22955,11 @@
       <c r="G534" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H534" s="6">
-        <f>"69' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H534" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">69' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I534" s="3" t="n"/>
       <c r="J534" s="3" t="n">
@@ -22471,9 +22997,14 @@
       <c r="G535" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H535" s="6">
-        <f>"62' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x45' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H535" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62' EF Z2 (127-140 bpm / 120-140 W) | 2x45' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I535" s="3" t="n"/>
       <c r="J535" s="3" t="n">
@@ -22641,9 +23172,14 @@
       <c r="G539" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H539" s="6">
-        <f>"84' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 6x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H539" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">84' EF (127-140 bpm / 120-140 W) | 6x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I539" s="3" t="n"/>
       <c r="J539" s="3" t="n">
@@ -22770,9 +23306,12 @@
       <c r="G542" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H542" s="6">
-        <f>"369' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x45' allure IM (136-146 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") dans la seconde moitié — r=10' Z2"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H542" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">369' Z2 (127-140 bpm / 120-140 W) dont 3x45' allure IM (136-146 bpm / 140-150 W) dans la seconde moitié — r=10' Z2
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I542" s="3" t="n"/>
       <c r="J542" s="3" t="n">
@@ -22976,9 +23515,11 @@
       <c r="G548" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H548" s="6">
-        <f>"69' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H548" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">69' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I548" s="3" t="n"/>
       <c r="J548" s="3" t="n">
@@ -23016,9 +23557,14 @@
       <c r="G549" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H549" s="6">
-        <f>"59' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x50' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement"&amp;CHAR(10)&amp;"FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H549" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">59' EF Z2 (127-140 bpm / 120-140 W) | 2x50' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=5'
+Objectif : spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
+FC bloc cible : 136-146 bpm (70-75% FC max) | Cadence : 85-92 rpm | RPE 5-6/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I549" s="3" t="n"/>
       <c r="J549" s="3" t="n">
@@ -23186,9 +23732,14 @@
       <c r="G553" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H553" s="6">
-        <f>"89' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 6x5' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H553" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">89' EF (127-140 bpm / 120-140 W) | 6x5' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I553" s="3" t="n"/>
       <c r="J553" s="3" t="n">
@@ -23315,9 +23866,12 @@
       <c r="G556" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H556" s="6">
-        <f>"386' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 3x50' allure IM (136-146 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") dans la seconde moitié — r=10' Z2"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H556" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">386' Z2 (127-140 bpm / 120-140 W) dont 3x50' allure IM (136-146 bpm / 140-150 W) dans la seconde moitié — r=10' Z2
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I556" s="3" t="n"/>
       <c r="J556" s="3" t="n">
@@ -23517,9 +24071,11 @@
       <c r="G562" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H562" s="6">
-        <f>"60' Z1 très facile (&lt; 127 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"&amp;") — récupération active"&amp;CHAR(10)&amp;"Cadence souple 85-90 rpm"</f>
-        <v/>
+      <c r="H562" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60' Z1 très facile (&lt; 127 bpm / 100-110 W) — récupération active
+Cadence souple 85-90 rpm</t>
+        </is>
       </c>
       <c r="I562" s="3" t="n"/>
       <c r="J562" s="3" t="n">
@@ -23557,9 +24113,14 @@
       <c r="G563" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H563" s="6">
-        <f>"35' EF Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 2x20' @ 88% FTP ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=5'"&amp;CHAR(10)&amp;"Objectif : garder du rythme pendant l'affûtage"&amp;CHAR(10)&amp;"FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H563" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35' EF Z2 (127-140 bpm / 120-140 W) | 2x20' @ 88% FTP (175 W) — r=5'
+Objectif : garder du rythme pendant l'affûtage
+FC bloc cible : ~159 bpm (82% FC max) | Cadence : 87-93 rpm | RPE 7-8/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I563" s="3" t="n"/>
       <c r="J563" s="3" t="n">
@@ -23726,9 +24287,14 @@
       <c r="G567" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H567" s="6">
-        <f>"35' EF (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x3' basse cadence (55-62 rpm) @ Z2 ("&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*85/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : force musculaire spécifique, économie de pédalage"&amp;CHAR(10)&amp;"FC : 131-155 bpm | RPE 6-7/10"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;90'"&amp;CHAR(10)&amp;"10' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H567" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35' EF (127-140 bpm / 120-140 W) | 3x3' basse cadence (55-62 rpm) @ Z2 (150-170 W) — r=3'
+Objectif : force musculaire spécifique, économie de pédalage
+FC : 131-155 bpm | RPE 6-7/10
+NUTRITION : 90g glucides/h si &gt;90'
+10' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I567" s="3" t="n"/>
       <c r="J567" s="3" t="n">
@@ -23856,9 +24422,12 @@
       <c r="G570" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H570" s="6">
-        <f>"120' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") dont 2x15' allure IM (136-146 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") dans la seconde moitié — r=10' Z2"&amp;CHAR(10)&amp;"Cadence 85-92 rpm"&amp;CHAR(10)&amp;"NUTRITION : 90g glucides/h si &gt;60'"</f>
-        <v/>
+      <c r="H570" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120' Z2 (127-140 bpm / 120-140 W) dont 2x15' allure IM (136-146 bpm / 140-150 W) dans la seconde moitié — r=10' Z2
+Cadence 85-92 rpm
+NUTRITION : 90g glucides/h si &gt;60'</t>
+        </is>
       </c>
       <c r="I570" s="3" t="n"/>
       <c r="J570" s="3" t="n">
@@ -23970,9 +24539,12 @@
       <c r="G574" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H574" s="6">
-        <f>"36' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x5' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=3'"&amp;CHAR(10)&amp;"Objectif : activation + vérification matériel (réglages, pression des pneus, ravitaillement de course)"&amp;CHAR(10)&amp;"3' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H574" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36' Z2 (127-140 bpm / 120-140 W) | 3x5' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=3'
+Objectif : activation + vérification matériel (réglages, pression des pneus, ravitaillement de course)
+3' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I574" s="3" t="n"/>
       <c r="J574" s="3" t="n">
@@ -24052,9 +24624,10 @@
       <c r="G576" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H576" s="6">
-        <f>"35' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — activation/vérification matériel"</f>
-        <v/>
+      <c r="H576" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35' Z2 très facile (127-140 bpm / 100-120 W) — activation/vérification matériel</t>
+        </is>
       </c>
       <c r="I576" s="3" t="n"/>
       <c r="J576" s="3" t="n">
@@ -24137,9 +24710,12 @@
       <c r="G578" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H578" s="6">
-        <f>"30' Z2 (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;") | 3x2' allure IM (136-146 bpm, 70-75% FC max / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"&amp;") — r=2'"&amp;CHAR(10)&amp;"Objectif : activation, retrouver les sensations de course"&amp;CHAR(10)&amp;"5' RC (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W"&amp;")"</f>
-        <v/>
+      <c r="H578" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30' Z2 (127-140 bpm / 120-140 W) | 3x2' allure IM (136-146 bpm, 70-75% FC max / 140-150 W) — r=2'
+Objectif : activation, retrouver les sensations de course
+5' RC (127-140 bpm / 120-140 W)</t>
+        </is>
       </c>
       <c r="I578" s="3" t="n"/>
       <c r="J578" s="3" t="n">
@@ -24305,9 +24881,10 @@
       <c r="G582" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H582" s="6">
-        <f>"25' Z2 très facile (127-140 bpm / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*50/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;" W"&amp;") — activation/vérification matériel"</f>
-        <v/>
+      <c r="H582" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25' Z2 très facile (127-140 bpm / 100-120 W) — activation/vérification matériel</t>
+        </is>
       </c>
       <c r="I582" s="3" t="n"/>
       <c r="J582" s="3" t="n">

</xml_diff>

<commit_message>
auto sync 2026-10-22 19:20:01
</commit_message>
<xml_diff>
--- a/Marathon_programme.xlsx
+++ b/Marathon_programme.xlsx
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="FTP">'Repères vélo'!$B$2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -86,7 +86,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 29' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 29' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -97,13 +97,13 @@
   </si>
   <si>
     <t>🎯 Sweet spot : travailler juste sous le seuil
-ÉCHAUFFEMENT — 20' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 20' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 22' à 180 W (91 % FTP) · 87-93 rpm · FC fin ≈165
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 22' à 190 W (91 % FTP) · 87-93 rpm · FC fin ≈165
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>Jeudi</t>
@@ -132,11 +132,11 @@
   </si>
   <si>
     <t>🎯 Force très légère, reprise
-ÉCHAUFFEMENT — 10' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 10' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -214,7 +214,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 38' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 38' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -225,13 +225,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 20' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 20' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 10' à 180 W (89 % FTP) · 87-93 rpm · FC fin ≈161
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 10' à 190 W (89 % FTP) · 87-93 rpm · FC fin ≈161
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>26' EF Z2 (127-140 bpm) | 4x20'' strides
@@ -245,11 +245,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 10' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 10' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -276,10 +276,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 156' (71.5 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 156' (71.5 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 40 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -318,7 +318,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 24' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 24' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -326,13 +326,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 20' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 20' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 9' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 9' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>Natation technique pré-course</t>
@@ -375,7 +375,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 33' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 33' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -383,13 +383,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 20' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 20' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 x :
-  • 9' à 185 W (92 % FTP) · 87-93 rpm · FC fin ≈167
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 9' à 195 W (92 % FTP) · 87-93 rpm · FC fin ≈167
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 195 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -431,10 +431,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 230' (106 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 230' (106 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 40 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -465,7 +465,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 52' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 52' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -473,13 +473,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 89' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 89' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 7' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 7' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -497,11 +497,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 39' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 39' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -539,7 +539,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 43' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 43' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -547,13 +547,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 45' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 45' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 x :
-  • 12' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 12' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>Natation test CSS 400/200</t>
@@ -578,11 +578,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 50' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 50' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -615,10 +615,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 236' (110 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 236' (110 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 40 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -652,12 +652,12 @@
   </si>
   <si>
     <t>🎯 Tolérance au lactate et relances, alternance sous / au-dessus du seuil
-ÉCHAUFFEMENT — 51' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 51' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 blocs de 12', chacun = 3 x (3' sous + 1' sur) enchaînés :
-  • 3' sous le seuil · 185 W (93 % FTP) · 87-93 rpm · FC ≈155
-  • 1' au-dessus · 215 W (107 % FTP) · FC ≈171
-  → 5' récup Z1 entre blocs · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 3' sous le seuil · 195 W (93 % FTP) · 87-93 rpm · FC ≈155
+  • 1' au-dessus · 225 W (107 % FTP) · FC ≈171
+  → 5' récup Z1 entre blocs · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 40 g glucides/h si &gt; 90'
 ⚠ Pilotage aux watts : sur le 1', la FC n'a pas le temps de suivre. Relance assise, sans à-coup</t>
   </si>
@@ -678,11 +678,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 61' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 61' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 40 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -713,10 +713,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 246' (115 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 246' (115 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 40 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -751,7 +751,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 43' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 43' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -762,14 +762,14 @@
   </si>
   <si>
     <t>🎯 Puissance aérobie maximale (VO2max), intervalles courts
-ÉCHAUFFEMENT — 40' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 ouvertures de 30'' à 240 W
+ÉCHAUFFEMENT — 40' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 ouvertures de 30'' à 250 W
 CORPS — 5 x :
-  • 3' à 230 W (115 % FTP) · 90-100 rpm · FC fin 184-194
-  • 3' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 34' Z2 · 120-140 W (60-70 % FTP), puis 10' souple &lt;110 W
+  • 3' à 240 W (115 % FTP) · 90-100 rpm · FC fin 184-194
+  • 3' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 34' Z2 · 125-145 W (60-70 % FTP), puis 10' souple &lt;115 W
 ⚡ RPE 8-9/10 · 🍌 40 g glucides/h si &gt; 90'
-⚠ Mode ERG. Si tu ne tiens plus 230 W sur la dernière, arrête une rép plus tôt : c'est la qualité qui compte</t>
+⚠ Mode ERG. Si tu ne tiens plus 240 W sur la dernière, arrête une rép plus tôt : c'est la qualité qui compte</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -789,11 +789,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 72' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 72' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 40 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -823,10 +823,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 257' (120 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 257' (120 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 40 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -844,7 +844,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 32' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 32' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -852,13 +852,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 32' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 32' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 15' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 15' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 50 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -877,11 +877,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 35' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 35' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -912,11 +912,11 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 167' (78 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 167' (78 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 📝 Semaine de décharge : volume réduit
 🍌 50 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S10 — 02/11/2026 → 08/11/2026   |     Phase 1 — Base</t>
@@ -948,15 +948,15 @@
   </si>
   <si>
     <t>🎯 Mesurer ta FTP (frais, après la semaine de décharge)
-ÉCHAUFFEMENT — 25' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 25' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
   dont 3 x 1' rapide à 110 rpm
-  puis 5' très facile · 100-120 W (50-60 % FTP)
+  puis 5' très facile · 105-125 W (50-60 % FTP)
 TEST — 20' effort maximal régulier · 85-95 rpm
-  • 5 premières minutes à 200 W (100 % FTP)
+  • 5 premières minutes à 210 W (100 % FTP)
   • puis +5 W toutes les 5' si tu te sens bien
   • note la puissance moyenne des 20' et la FC moyenne des 10 dernières minutes
-APRÈS LE TEST — 56' Z2 · 120-140 W (60-70 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+APRÈS LE TEST — 56' Z2 · 125-145 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 🧮 FTP = 0,95 × puissance moyenne des 20' → à reporter dans l'onglet Repères vélo (je recale ensuite les watts du plan)
 ⚡ RPE 9/10 · 🍌 50 g glucides/h si &gt; 90'
 ⚠ Mode libre (pas d'ERG) : pars prudent, c'est la régularité qui fait le bon test</t>
@@ -979,11 +979,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 70' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 70' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 50 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1013,10 +1013,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 261' (122 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 261' (122 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 50 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1056,13 +1056,13 @@
   </si>
   <si>
     <t>🎯 Élever le seuil (blocs courts à intensité haute)
-ÉCHAUFFEMENT — 64' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 64' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 4 x :
-  • 9' à 205 W (102 % FTP) · 88-95 rpm · FC fin ≈169
-  • 4' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 9' à 215 W (102 % FTP) · 88-95 rpm · FC fin ≈169
+  • 4' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 8/10 · 🍌 50 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 205 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 215 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1081,11 +1081,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 72' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 72' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 50 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1116,10 +1116,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 268' (125 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 268' (125 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 50 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1150,7 +1150,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 47' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 47' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -1158,12 +1158,12 @@
   </si>
   <si>
     <t>🎯 Tolérance au lactate et relances, alternance sous / au-dessus du seuil
-ÉCHAUFFEMENT — 71' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 71' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 blocs de 20', chacun = 5 x (3' sous + 1' sur) enchaînés :
-  • 3' sous le seuil · 185 W (93 % FTP) · 87-93 rpm · FC ≈155
-  • 1' au-dessus · 215 W (107 % FTP) · FC ≈171
-  → 5' récup Z1 entre blocs · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 3' sous le seuil · 195 W (93 % FTP) · 87-93 rpm · FC ≈155
+  • 1' au-dessus · 225 W (107 % FTP) · FC ≈171
+  → 5' récup Z1 entre blocs · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 50 g glucides/h si &gt; 90'
 ⚠ Pilotage aux watts : sur le 1', la FC n'a pas le temps de suivre. Relance assise, sans à-coup</t>
   </si>
@@ -1185,11 +1185,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 74' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 74' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 50 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1221,10 +1221,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 274' (128 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 274' (128 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 50 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1258,13 +1258,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 30' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 30' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 18' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 18' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 60 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Technique, puis allure IM en continu
@@ -1287,11 +1287,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 42' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 42' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1315,11 +1315,11 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 182' (85 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 182' (85 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 📝 Semaine de décharge : volume réduit
 🍌 60 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S14 — 30/11/2026 → 06/12/2026   |     Phase 2 — Build</t>
@@ -1343,13 +1343,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 61' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 61' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 25' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 25' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 60 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Seuil (CSS) puis allure soutenue
@@ -1375,11 +1375,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 74' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 74' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 60 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1411,10 +1411,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 279' (130 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 279' (130 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 60 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1451,14 +1451,14 @@
   </si>
   <si>
     <t>🎯 Puissance aérobie maximale (VO2max), intervalles courts
-ÉCHAUFFEMENT — 40' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 ouvertures de 30'' à 240 W
+ÉCHAUFFEMENT — 40' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 ouvertures de 30'' à 250 W
 CORPS — 5 x :
-  • 4' à 225 W (112 % FTP) · 90-100 rpm · FC fin 184-194
-  • 4' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 51' Z2 · 120-140 W (60-70 % FTP), puis 10' souple &lt;110 W
+  • 4' à 235 W (112 % FTP) · 90-100 rpm · FC fin 184-194
+  • 4' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 51' Z2 · 125-145 W (60-70 % FTP), puis 10' souple &lt;115 W
 ⚡ RPE 8-9/10 · 🍌 60 g glucides/h si &gt; 90'
-⚠ Mode ERG. Si tu ne tiens plus 225 W sur la dernière, arrête une rép plus tôt : c'est la qualité qui compte</t>
+⚠ Mode ERG. Si tu ne tiens plus 235 W sur la dernière, arrête une rép plus tôt : c'est la qualité qui compte</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1478,11 +1478,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 79' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 79' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 60 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1514,10 +1514,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 285' (133 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 285' (133 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 60 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1551,7 +1551,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 51' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 51' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -1559,11 +1559,11 @@
   </si>
   <si>
     <t>🎯 Endurance de tempo, pont vers l'allure IM
-ÉCHAUFFEMENT — 66' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 66' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 x :
-  • 20' tempo · 165-175 W (82-87 % FTP) · 85-92 rpm · FC 147-159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 20' tempo · 175-185 W (82-87 % FTP) · 85-92 rpm · FC 147-159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 60 g glucides/h si &gt; 90'
 ⚠ Mode ERG. Bloc régulier : si la FC dépasse 159, baisse de 5 W</t>
   </si>
@@ -1585,11 +1585,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 83' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 83' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 60 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1621,10 +1621,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 289' (135 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 289' (135 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 60 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -1647,13 +1647,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 70' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 70' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 12' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 12' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 60 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Technique, puis allure IM en continu
@@ -1674,10 +1674,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale
-CORPS — 100' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 100' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
 📝 Parcours Paris, terrain plat
 🍌 60 g glucides/h si &gt; 90'
-⚠ Plafond 140 bpm ; dans les bosses, max 170 W</t>
+⚠ Plafond 140 bpm ; dans les bosses, max 180 W</t>
   </si>
   <si>
     <t>🎯 Progression SV1 → SV2, endurance de seuil
@@ -1780,7 +1780,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 60' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 60' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -1788,10 +1788,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 193' (90 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 193' (90 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 60 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 15'</t>
@@ -1830,13 +1830,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 53' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 53' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 28' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 28' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 70 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>EF Z2</t>
@@ -1865,11 +1865,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 61' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 61' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1898,10 +1898,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 257' (120 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 257' (120 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 70 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>Natation récupération</t>
@@ -1924,11 +1924,11 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 56' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 56' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 30' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 30' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
@@ -1949,11 +1949,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 65' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 65' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -1981,10 +1981,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 279' (130 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 279' (130 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 70 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 20'</t>
@@ -2023,7 +2023,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 54' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 54' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -2031,13 +2031,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 62' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 62' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 30' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 30' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 70 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>71' EF Z2 (127-140 bpm)
@@ -2058,11 +2058,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 72' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 72' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2094,10 +2094,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 296' (138 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 296' (138 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 70 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -2131,7 +2131,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 39' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 39' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -2139,13 +2139,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 35' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 35' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 20' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 20' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 70 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>46' EF Z2 (127-140 bpm) | 4x20'' strides
@@ -2163,11 +2163,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 40' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 40' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2191,11 +2191,11 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 193' (90 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 193' (90 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 📝 Semaine de décharge : volume réduit
 🍌 70 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S23 — 01/02/2027 → 07/02/2027   |     Phase 3 — Pré-IM</t>
@@ -2214,15 +2214,15 @@
   </si>
   <si>
     <t>🎯 Mesurer ta FTP (frais, après la semaine de décharge)
-ÉCHAUFFEMENT — 25' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 25' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
   dont 3 x 1' rapide à 110 rpm
-  puis 5' très facile · 100-120 W (50-60 % FTP)
+  puis 5' très facile · 105-125 W (50-60 % FTP)
 TEST — 20' effort maximal régulier · 85-95 rpm
-  • 5 premières minutes à 200 W (100 % FTP)
+  • 5 premières minutes à 210 W (100 % FTP)
   • puis +5 W toutes les 5' si tu te sens bien
   • note la puissance moyenne des 20' et la FC moyenne des 10 dernières minutes
-APRÈS LE TEST — 81' Z2 · 120-140 W (60-70 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+APRÈS LE TEST — 81' Z2 · 125-145 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 🧮 FTP = 0,95 × puissance moyenne des 20' → à reporter dans l'onglet Repères vélo (je recale ensuite les watts du plan)
 ⚡ RPE 9/10 · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Mode libre (pas d'ERG) : pars prudent, c'est la régularité qui fait le bon test</t>
@@ -2244,11 +2244,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 74' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 74' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2280,10 +2280,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 300' (140 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 300' (140 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 70 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S24 — 08/02/2027 → 14/02/2027   |     Phase 3 — WE Paris 13/02</t>
@@ -2302,7 +2302,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 56' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 56' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -2324,14 +2324,14 @@
   </si>
   <si>
     <t>🎯 Puissance aérobie maximale (VO2max), intervalles courts
-ÉCHAUFFEMENT — 40' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 ouvertures de 30'' à 240 W
+ÉCHAUFFEMENT — 40' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 ouvertures de 30'' à 250 W
 CORPS — 6 x :
-  • 4' à 225 W (112 % FTP) · 90-100 rpm · FC fin 184-194
-  • 4' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 56' Z2 · 120-140 W (60-70 % FTP), puis 10' souple &lt;110 W
+  • 4' à 235 W (112 % FTP) · 90-100 rpm · FC fin 184-194
+  • 4' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 56' Z2 · 125-145 W (60-70 % FTP), puis 10' souple &lt;115 W
 ⚡ RPE 8-9/10 · 🍌 70 g glucides/h si &gt; 90'
-⚠ Mode ERG. Si tu ne tiens plus 225 W sur la dernière, arrête une rép plus tôt : c'est la qualité qui compte</t>
+⚠ Mode ERG. Si tu ne tiens plus 235 W sur la dernière, arrête une rép plus tôt : c'est la qualité qui compte</t>
   </si>
   <si>
     <t>89' EF Z2 (127-140 bpm)
@@ -2349,11 +2349,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 80' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 80' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 70 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2370,10 +2370,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 311' (145 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 311' (145 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 70 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S25 — 15/02/2027 → 21/02/2027   |     Phase 4 — Spécifique IM</t>
@@ -2396,7 +2396,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 58' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 58' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -2404,13 +2404,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 78' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 78' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 33' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 33' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 80 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>83' EF Z2 (127-140 bpm)
@@ -2431,11 +2431,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 89' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 89' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 80 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2466,10 +2466,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 321' (150 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 321' (150 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 80 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 25'</t>
@@ -2510,11 +2510,11 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 72' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 72' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 40' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 40' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 80 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
@@ -2535,11 +2535,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 95' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 95' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 80 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2571,10 +2571,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 332' (155 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 332' (155 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 80 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -2635,10 +2635,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale
-CORPS — 120' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 120' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
 📝 Pas de bloc FTP cette semaine (reprise post-ski)
 🍌 80 g glucides/h si &gt; 90'
-⚠ Plafond 140 bpm ; dans les bosses, max 170 W</t>
+⚠ Plafond 140 bpm ; dans les bosses, max 180 W</t>
   </si>
   <si>
     <t>68' EF Z2 (127-140 bpm)
@@ -2660,10 +2660,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale
-CORPS — 96' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 96' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 📝 Pas de travail de force cette semaine
 🍌 80 g glucides/h si &gt; 90'
-⚠ Plafond 140 bpm ; dans les bosses, max 170 W</t>
+⚠ Plafond 140 bpm ; dans les bosses, max 180 W</t>
   </si>
   <si>
     <t>🎯 Technique, puis allure IM en continu
@@ -2686,10 +2686,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 246' (115 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 246' (115 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 80 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -2705,13 +2705,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 66' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 66' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 30' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 30' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 80 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Test CSS : mesurer ton allure seuil
@@ -2732,11 +2732,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 77' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 77' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 80 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2764,10 +2764,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 300' (140 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 300' (140 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 80 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -2801,13 +2801,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 52' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 52' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 20' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 20' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 80 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>65' EF Z2 (127-140 bpm) | 4x20'' strides
@@ -2826,11 +2826,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 46' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 46' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2855,11 +2855,11 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 236' (110 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 236' (110 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 📝 Semaine de décharge : volume réduit
 🍌 80 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -2887,11 +2887,11 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 61' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 61' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 x :
-  • 25' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 25' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 80 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
@@ -2913,11 +2913,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 79' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 79' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 80 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -2955,13 +2955,13 @@
   </si>
   <si>
     <t>🎯 Travailler juste sous le seuil lactique (sweet spot)
-ÉCHAUFFEMENT — 106' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 106' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 25' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 25' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 90 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -2976,11 +2976,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 86' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 86' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3011,10 +3011,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 343' (160 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 343' (160 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 30'</t>
@@ -3038,11 +3038,11 @@
   </si>
   <si>
     <t>🎯 Endurance de tempo, pont vers l'allure IM
-ÉCHAUFFEMENT — 100' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 100' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 x :
-  • 20' tempo · 165-175 W (82-87 % FTP) · 85-92 rpm · FC 147-159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 20' tempo · 175-185 W (82-87 % FTP) · 85-92 rpm · FC 147-159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Mode ERG. Bloc régulier : si la FC dépasse 159, baisse de 5 W</t>
   </si>
@@ -3064,11 +3064,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 99' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 99' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 5 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3099,10 +3099,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 364' (170 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  Puissance normalisée visée ≤ 140 W (IF ≤ 0,70)
+CORPS — 364' (170 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  Puissance normalisée visée ≤ 145 W (IF ≤ 0,70)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 35'</t>
@@ -3135,13 +3135,13 @@
   </si>
   <si>
     <t>🎯 Rester juste sous le seuil lactique, séance complète — Lacanau est une course en Z3, pas d'affûtage
-ÉCHAUFFEMENT — 67' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 67' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 25' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 25' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · 🍌 90 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -3159,11 +3159,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 26' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 26' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 3 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3192,7 +3192,7 @@
   </si>
   <si>
     <t>🎯 Vérification matériel / dépôt sac T1-T2
-CORPS — 15' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 15' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Aucun effort : on vérifie le vélo, pas la forme</t>
   </si>
   <si>
@@ -3221,10 +3221,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale
-CORPS — 118' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 118' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
 📝 Z2 facile, pas de bloc FTP (reprise post-Lacanau)
 🍌 90 g glucides/h si &gt; 90'
-⚠ Plafond 140 bpm ; dans les bosses, max 170 W</t>
+⚠ Plafond 140 bpm ; dans les bosses, max 180 W</t>
   </si>
   <si>
     <t>🎯 Endurance aérobie, allure régulière
@@ -3246,8 +3246,8 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale
-CORPS — 75' Z2 facile · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
-⚠ Plafond 140 bpm ; dans les bosses, max 170 W</t>
+CORPS — 75' Z2 facile · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-90 rpm
+⚠ Plafond 140 bpm ; dans les bosses, max 180 W</t>
   </si>
   <si>
     <t>🎯 Technique, puis allure IM en continu
@@ -3268,10 +3268,10 @@
   </si>
   <si>
     <t>🎯 Endurance fondamentale, tenir la durée
-CORPS — 214' (100 km) en Z2 · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-92 rpm
+CORPS — 214' (100 km) en Z2 · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-92 rpm
 📝 Z2 léger, reprise du volume
 🍌 90 g glucides/h si &gt; 90'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>Z2 92' — allure conversationnelle
@@ -3304,13 +3304,13 @@
   </si>
   <si>
     <t>🎯 Reprendre le développement du seuil (FTP)
-ÉCHAUFFEMENT — 85' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 85' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 25' à 180 W (90 % FTP) · 87-93 rpm · FC fin ≈163
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 25' à 190 W (90 % FTP) · 87-93 rpm · FC fin ≈163
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 90 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 180 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 190 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>47' EF Z1-Z2 (120-135 bpm) — COURT
@@ -3318,11 +3318,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 87' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 87' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3345,11 +3345,11 @@
   </si>
   <si>
     <t>🎯 Spécificité IM : allure de course dans la fatigue
-CORPS — 321' (150 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 2 x 30' allure IM · 140-150 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 321' (150 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 2 x 30' allure IM · 145-160 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>🎯 Récupération : relâchement et amplitude
@@ -3383,11 +3383,11 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 69' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 69' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 35' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 35' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
@@ -3401,11 +3401,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 74' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 74' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 6 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3433,11 +3433,11 @@
   </si>
   <si>
     <t>🎯 Spécificité IM : allure de course dans la fatigue
-CORPS — 343' (160 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 x 30' allure IM · 140-150 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 343' (160 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 x 30' allure IM · 145-160 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S38 — 17/05/2027 → 23/05/2027   |     Phase 4 — Spécifique IM (Deload + Grand Brick)</t>
@@ -3462,13 +3462,13 @@
   </si>
   <si>
     <t>🎯 Développer la puissance au seuil (FTP)
-ÉCHAUFFEMENT — 33' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 33' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 22' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 22' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 90 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>52' EF Z2 (127-140 bpm) | 4x20'' strides
@@ -3487,11 +3487,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 42' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 42' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 4 x :
-  • 4' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 4' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3514,9 +3514,9 @@
   </si>
   <si>
     <t>🎯 Grand Brick : répétition générale du jour J (vélo, 2/3)
-CORPS — 300' en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 x 40' allure IM · 140-150 W (70-75 % FTP) · FC 136-146
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 300' en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 x 40' allure IM · 145-160 W (70-75 % FTP) · FC 136-146
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h
 ⚠ Stratégie course complète : nutrition, position, tenue et matériel du jour J</t>
   </si>
@@ -3541,7 +3541,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 64' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 64' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -3559,21 +3559,21 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 53' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 53' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 3 x :
-  • 30' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 30' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 78' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 78' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 6 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3603,11 +3603,11 @@
   </si>
   <si>
     <t>🎯 Spécificité IM : allure de course dans la fatigue
-CORPS — 354' (165 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 x 40' allure IM · 140-150 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 354' (165 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 x 40' allure IM · 145-160 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S40 — 31/05/2027 → 06/06/2027   |     Phase 4 — Bloc Final IM</t>
@@ -3634,7 +3634,7 @@
   </si>
   <si>
     <t>🎯 Récupération active
-CORPS — 69' Z1 très facile · 100-110 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
+CORPS — 69' Z1 très facile · 105-115 W (50-55 % FTP) · &lt;127 bpm · 85-90 rpm
 ⚠ Zéro effort, jambes qui tournent : si tu hésites, encore plus facile</t>
   </si>
   <si>
@@ -3642,21 +3642,21 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 62' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 62' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 45' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 45' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 84' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 84' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 6 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3687,11 +3687,11 @@
   </si>
   <si>
     <t>🎯 Spécificité IM : allure de course dans la fatigue
-CORPS — 369' (172 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 x 45' allure IM · 140-150 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 369' (172 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 x 45' allure IM · 145-160 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 40'</t>
@@ -3729,11 +3729,11 @@
   </si>
   <si>
     <t>🎯 Spécificité Ironman : rouler à l'effort de course et répéter le ravitaillement
-ÉCHAUFFEMENT — 59' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 59' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 50' allure IM · 140-150 W (70-75 % FTP) · 85-92 rpm · FC 136-146
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 50' allure IM · 145-160 W (70-75 % FTP) · 85-92 rpm · FC 136-146
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 5-6/10 · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Position aéro tenue tout le bloc, et ravitaillement pris comme en course : c'est la répétition du jour J</t>
   </si>
@@ -3754,11 +3754,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 89' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 89' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 6 x :
-  • 5' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 5' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3789,11 +3789,11 @@
   </si>
   <si>
     <t>🎯 Spécificité IM : allure de course dans la fatigue
-CORPS — 386' (180 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 3 x 50' allure IM · 140-150 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 386' (180 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 3 x 50' allure IM · 145-160 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t>CAP en Brick — 45'</t>
@@ -3819,13 +3819,13 @@
   </si>
   <si>
     <t>🎯 Garder du rythme pendant l'affûtage
-ÉCHAUFFEMENT — 35' Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+ÉCHAUFFEMENT — 35' Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
 CORPS — 2 x :
-  • 20' à 175 W (88 % FTP) · 87-93 rpm · FC fin ≈159
-  • 5' récup Z1 · &lt;110 W (&lt;55 % FTP)
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+  • 20' à 185 W (88 % FTP) · 87-93 rpm · FC fin ≈159
+  • 5' récup Z1 · &lt;115 W (&lt;55 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 7-8/10 · 🍌 90 g glucides/h si &gt; 90'
-⚠ Mode ERG. Ne pars jamais au-dessus de 175 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
+⚠ Mode ERG. Ne pars jamais au-dessus de 185 W ; la FC qui dérive en fin de bloc est normale, ce sont les watts qui commandent</t>
   </si>
   <si>
     <t>60' EF Z2 (127-140 bpm)
@@ -3843,11 +3843,11 @@
   </si>
   <si>
     <t>🎯 Force musculaire spécifique, économie de pédalage
-ÉCHAUFFEMENT — 35' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 35' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 3 x :
-  • 3' basse cadence · 150-170 W (75-85 % FTP) · 55-62 rpm
+  • 3' basse cadence · 160-180 W (75-85 % FTP) · 55-62 rpm
   • 3' récup Z2 souple · 90 rpm
-RETOUR AU CALME — 10' Z2 souple · 120-140 W (60-70 % FTP)
+RETOUR AU CALME — 10' Z2 souple · 125-145 W (60-70 % FTP)
 ⚡ RPE 6-7/10 · FC 131-155 normale sur les blocs · 🍌 90 g glucides/h si &gt; 90'
 ⚠ Assis, buste immobile, genou dans l'axe : c'est la jambe qui pousse, pas le dos</t>
   </si>
@@ -3879,11 +3879,11 @@
   </si>
   <si>
     <t>🎯 Spécificité IM : allure de course dans la fatigue
-CORPS — 120' (56 km) en Z2 · 120-140 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
-  dont 2 x 15' allure IM · 140-150 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
-  Puissance normalisée visée ≤ 145 W (IF ≤ 0,72)
+CORPS — 120' (56 km) en Z2 · 125-145 W (60-70 % FTP) · &lt;140 bpm · 85-92 rpm
+  dont 2 x 15' allure IM · 145-160 W (70-75 % FTP) · FC 136-146 dans la seconde moitié — 10' Z2 entre les blocs
+  Puissance normalisée visée ≤ 150 W (IF ≤ 0,72)
 🍌 90 g glucides/h si &gt; 60'
-⚠ Dans les bosses, plafond 170 W : on monte en Z2-Z3, jamais au seuil</t>
+⚠ Dans les bosses, plafond 180 W : on monte en Z2-Z3, jamais au seuil</t>
   </si>
   <si>
     <t xml:space="preserve">  S43 — 21/06/2027 → 27/06/2027   |     COMPETITION — IRONMAN LES SABLES D'OLONNE 27/06</t>
@@ -3899,12 +3899,12 @@
   </si>
   <si>
     <t>🎯 Activation + vérification matériel (réglages, pression des pneus, ravitaillement de course)
-ÉCHAUFFEMENT — 36' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 36' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 3 x :
-  • 5' allure IM · 140-150 W (70-75 % FTP) · FC 136-146
-  • 3' souple · &lt;110 W (&lt;55 % FTP)
+  • 5' allure IM · 145-160 W (70-75 % FTP) · FC 136-146
+  • 3' souple · &lt;115 W (&lt;55 % FTP)
 RETOUR AU CALME — 3' souple
-⚠ Sensations seulement : aucun watt au-dessus de 150 W, on garde tout pour dimanche</t>
+⚠ Sensations seulement : aucun watt au-dessus de 160 W, on garde tout pour dimanche</t>
   </si>
   <si>
     <t>20' EF Z2 (127-140 bpm) | 4x20'' strides en fin
@@ -3915,7 +3915,7 @@
   </si>
   <si>
     <t>🎯 Activation/vérification matériel
-CORPS — 35' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 35' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Aucun effort : on vérifie le vélo, pas la forme</t>
   </si>
   <si>
@@ -3938,12 +3938,12 @@
   </si>
   <si>
     <t>🎯 Activation, retrouver les sensations de course
-ÉCHAUFFEMENT — 30' Z2 · 120-140 W (60-70 % FTP) · 85-92 rpm
+ÉCHAUFFEMENT — 30' Z2 · 125-145 W (60-70 % FTP) · 85-92 rpm
 CORPS — 3 x :
-  • 2' allure IM · 140-150 W (70-75 % FTP) · FC 136-146
-  • 2' souple · &lt;110 W (&lt;55 % FTP)
+  • 2' allure IM · 145-160 W (70-75 % FTP) · FC 136-146
+  • 2' souple · &lt;115 W (&lt;55 % FTP)
 RETOUR AU CALME — 5' souple
-⚠ Sensations seulement : aucun watt au-dessus de 150 W, on garde tout pour dimanche</t>
+⚠ Sensations seulement : aucun watt au-dessus de 160 W, on garde tout pour dimanche</t>
   </si>
   <si>
     <t>EF + 3x1' allure IM + visualisation</t>
@@ -3974,7 +3974,7 @@
   </si>
   <si>
     <t>🎯 Activation/vérification matériel
-CORPS — 25' Z2 très facile · 100-120 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
+CORPS — 25' Z2 très facile · 105-125 W (50-60 % FTP) · &lt;140 bpm · 85-90 rpm
 ⚠ Aucun effort : on vérifie le vélo, pas la forme</t>
   </si>
   <si>
@@ -4985,7 +4985,7 @@
     <t>FTP actuelle (W)</t>
   </si>
   <si>
-    <t>← à modifier après les tests FTP de S10 et S23 : ce tableau se recalcule. Dans les séances du plan, les watts sont écrits pour 200 W ; le % FTP indiqué à côté reste la référence (watts à recaler après chaque test)</t>
+    <t>← à modifier après les tests FTP de S10 et S23 : ce tableau se recalcule. Dans les séances du plan, les watts sont écrits pour 210 W (FTP de travail estimée au ressenti le 22/10/2026, à remplacer par la FTP mesurée au test de S10) ; le % FTP indiqué à côté reste la référence (watts à recaler après chaque test)</t>
   </si>
   <si>
     <t>% FTP</t>
@@ -26444,7 +26444,7 @@
         <v>922</v>
       </c>
       <c r="B2" s="144">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C2" s="176" t="s">
         <v>923</v>
@@ -26484,7 +26484,7 @@
       </c>
       <c r="E4" s="143" t="str">
         <f>"&lt; "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*55/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>&lt; 110 W</v>
+        <v>&lt; 115 W</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26502,7 +26502,7 @@
       </c>
       <c r="E5" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*56/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W (cible "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*60/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;" W)"</f>
-        <v>110-150 W (cible 120-140 W)</v>
+        <v>120-160 W (cible 125-145 W)</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26520,7 +26520,7 @@
       </c>
       <c r="E6" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*70/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*75/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>140-150 W</v>
+        <v>145-160 W</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26538,7 +26538,7 @@
       </c>
       <c r="E7" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*76/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*87/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>150-175 W</v>
+        <v>160-185 W</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26556,7 +26556,7 @@
       </c>
       <c r="E8" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*88/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*94/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>175-190 W</v>
+        <v>185-195 W</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26574,7 +26574,7 @@
       </c>
       <c r="E9" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*95/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*105/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>190-210 W</v>
+        <v>200-220 W</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26592,7 +26592,7 @@
       </c>
       <c r="E10" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*93/500,0)*5,"0"),"?")&amp;" / "&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*107/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>185 / 215 W</v>
+        <v>195 / 225 W</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26610,7 +26610,7 @@
       </c>
       <c r="E11" s="143" t="str">
         <f>IF(FTP&gt;0,TEXT(ROUND(FTP*106/500,0)*5,"0"),"?")&amp;"-"&amp;IF(FTP&gt;0,TEXT(ROUND(FTP*120/500,0)*5,"0"),"?")&amp;" W"</f>
-        <v>210-240 W</v>
+        <v>225-250 W</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>